<commit_message>
debug: 添加 Agent 请求日志 + 清理 pycache + --reload 模式
- agent_router.py: 记录每条 chat 请求的 msg 和 history
- 清理所有 __pycache__ 确保加载最新 Python 代码
- uvicorn 改用 --reload 自动重载
</commit_message>
<xml_diff>
--- a/backend/data/别墅装修_最新.xlsx
+++ b/backend/data/别墅装修_最新.xlsx
@@ -3018,7 +3018,7 @@
       </c>
       <c r="M18" s="46" t="inlineStr">
         <is>
-          <t>已支付</t>
+          <t>未开始</t>
         </is>
       </c>
       <c r="N18" s="47" t="inlineStr">
@@ -3027,7 +3027,7 @@
         </is>
       </c>
       <c r="O18" t="n">
-        <v>80000</v>
+        <v>0</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -3178,7 +3178,11 @@
       <c r="P20" t="n">
         <v>0</v>
       </c>
-      <c r="Q20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>待补充</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="42" customHeight="1" s="184">
       <c r="A21" s="43" t="inlineStr">

</xml_diff>